<commit_message>
chore(scrape): auto update 2026-05-07 17:11 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -509,8 +509,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>大阪府副業・兼業人材活用促進補助金</t>
@@ -674,7 +672,6 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>開催概要 大阪市は、脱炭素社会「ゼロカーボン おおさか」の実現に向けた取組を進めています。このたび、連携協定を締結している三井住友海上火災保険株式会社と株式会社バイウィルとともに、脱炭素をテーマとしたセミナー「知れば得する！脱炭素経営×補助金活用 企業が未来を創るセミナー」を開催します。本セミナーでは、脱炭素に関する最新の動向や、本市の支援策、企業における実践例など、今後の脱炭素経営に役立つ情報をご提供します。 1 日時 令和8年2月…</t>
@@ -707,7 +704,6 @@
           <t>公募開始</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>上限300万円</t>
@@ -745,7 +741,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>500万円</t>
@@ -783,7 +778,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>限度額300万円</t>
@@ -821,7 +815,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>限度額10万円</t>
@@ -859,7 +852,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>限度額とします。 補助限度額：300万円</t>
@@ -939,8 +931,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>東大阪市 東大阪市障害者雇用奨励金 ▶東大阪市障害者雇用奨励金 （別ウインドウで開く） 市内在住の障害者を市内の事業所において常用雇用労働者として雇用する事業主の方に対し、障害者の雇用促進を目的として、障害者雇用奨励金を支給しています。 問合せ先：労働雇用政策室(06-4309-3178) 東大阪市トライアル雇用支援金 ▶東大阪市トライアル雇用支援金 （別ウインドウで開く） 若年者等の雇用を促進するため、国(ハローワーク)のトライアル…</t>
@@ -973,8 +963,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>東大阪市では、市内中小企業者又は市内中小企業者2社以上が共同して行う 新たな技術の研究や新製品の開発に向けた取り組み 及び市内中小企業を中心に構成する企業グループが行う 経営力の向上に資する調査研究や講習会 の開催に対して助成金を交付いたします。 備考：助成金の交付にあたっては、事業計画等をご提案いただき審査会の採択を受ける必要がございます。 当助成金の詳しい内容は 公益財団法人東大阪市産業創造勤労者支援機構 (別のサイトへ移動します…</t>
@@ -1007,8 +995,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>東大阪市では、市内製造業の新技術・新製品に関する特許権の「保護」及び「権利化」を促進させるため、出願審査請求に直接必要となる経費に対して補助金を交付しています。 当補助金の詳しい内容は 公益財団法人東大阪市産業創造勤労者支援機構(別のサイトへ移動します) をご覧ください。</t>
@@ -1041,8 +1027,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>ページ番号1018028 補助金・融資・相談等 企業支援・産業振興に関するイベント・セミナー 産業振興のための施策 市内商工業や商店街イベントについての情報発信 吹田市ふるさと納税 工場立地・小売店舗出店に係る届け出 このページに関する お問い合わせ 都市魅力部 地域経済振興室 〒564-8550 大阪府吹田市泉町1丁目3番40号（低層棟3階316番窓口、高層棟7階706番窓口） 電話番号： 【庶務】 06-6384-1356 【企業…</t>
@@ -1075,8 +1059,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>ページ番号1018029 起業・創業 事業者向けの補助金 商店街向けの補助金 税制優遇制度 中小企業向けの融資制度 事業承継支援 相談制度 ご意見をお聞かせください このページに問題点はありましたか？（複数回答可） 特にない 内容が分かりにくい ページを探しにくい 情報が少ない 文章量が多い 送信</t>
@@ -1151,7 +1133,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>上限） 20万円</t>
@@ -1357,7 +1338,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>上限額500万円</t>
@@ -1395,7 +1375,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>上限額500万円</t>
@@ -1475,8 +1454,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>ページ番号1018058 地元企業等共同研究開発事業補助金の直近5年分の交付実績を公開しています。 令和6年度 地元企業等共同研究開発事業補助金 交付実績 令和5年度 地元企業等共同研究開発事業補助金 交付実績 令和4年度 地元企業等共同研究開発事業補助金 交付実績 令和3年度 地元企業等共同研究開発事業補助金 交付実績 令和2年度 地元企業等共同研究開発事業補助金 交付実績 このページに関する お問い合わせ 都市魅力部 地域経済振興…</t>
@@ -1509,8 +1486,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>ページ番号1021242 商店街活性化のための補助 商店街等の空き店舗活用事業 ご意見をお聞かせください このページに問題点はありましたか？（複数回答可） 特にない 内容が分かりにくい ページを探しにくい 情報が少ない 文章量が多い 送信</t>
@@ -1543,7 +1518,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>上限300万円</t>
@@ -1581,7 +1555,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>補助上限が20万円</t>
@@ -1619,7 +1592,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>限度額15万円</t>
@@ -1783,7 +1755,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>上限10万円</t>
@@ -1863,7 +1834,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>補助上限額：30万円</t>
@@ -1901,7 +1871,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>補助上限額：10万円</t>
@@ -1939,7 +1908,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>補助上限： 10万円</t>
@@ -2103,7 +2071,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>上限】1億円</t>
@@ -2141,7 +2108,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>上限 300万円</t>
@@ -2179,7 +2145,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>上限 500万円</t>
@@ -2217,7 +2182,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>上限 250万円</t>
@@ -2255,8 +2219,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>令和6年度豊中市チャレンジ事業補助金の申込受付は終了しました</t>
@@ -2289,7 +2251,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>上限額：30万円</t>
@@ -2369,8 +2330,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>本文 建築物の耐震化（補助金等） お知らせ 2026年4月1日更新 耐震診断・改修事業者情報提供制度 制度・事業等 2026年4月1日更新 木造住宅耐震事業費用の補助制度 2026年4月1日更新 木造住宅除却工事補助制度補助 2023年3月31日更新 分譲マンションの耐震補助制度 2023年3月31日更新 （木造以外）耐震診断費用の補助制度 手続き 2022年3月30日更新 耐震事業者のみなさまへ 計画 2026年4月1日更新 高槻市…</t>
@@ -2403,8 +2362,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>本文 ブロック塀等の安全確保（補助金等） お知らせ 2026年4月1日更新 ブロック塀撤去事業者の情報提供 2022年3月22日更新 塀の安全点検 制度・事業等 2025年4月1日更新 ブロック塀等撤去工事費の補助制度 2022年3月22日更新 高槻市ブロック塀等の安全確保に向けた手引き</t>
@@ -2437,7 +2394,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>15,000,000円</t>
@@ -2517,8 +2473,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>神戸市では、市内中小企業の操業基盤の強化を図るため、技術力や生産性の向上、受注拡大、研究開発機能の強化などに向けた設備投資等を行う事業者を対象とする助成制度を実施しています。 2026年度 神戸市中小企業投資促進等助成制度 【参考】 2025年度 神戸市中小企業投資促進等助成制度 2024年度 神戸市中小企業投資促進等助成制度 2023年度 神戸市中小企業投資促進等助成制度 2022年度(令和4年度) 神戸市中小製造業投資促進等助成制…</t>
@@ -2551,8 +2505,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>神戸市では、戦略産業分野における新事業展開のための試作開発や新素材・新製品の実用化に向けた開発、大学・公設試等の研究機関等と連携し社会課題の解決につながる革新的な開発に取り組む神戸市内中小企業若しくは神戸市内中小企業等により構成されるコンソーシアムに対し補助金を交付することにより、ものづくり技術の高度化と市内産業の振興を図ることを目的としています。 2025年度「神戸挑戦企業等支援補助制度」 （参考） 2024年度「神戸挑戦企業等支援…</t>
@@ -2585,8 +2537,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>神戸市では、水素関連製品の実用化に向けた研究・開発・実証に取り組む、神戸市内の中小企業若しくは神戸市内の中小企業等より構成されるコンソーシアムを対象とする補助制度を実施しています。 2025年度 水素関連製品の研究・開発・実証補助金 （参考） 2024年度 水素関連製品の研究・開発・実証補助金 2023年度 水素関連製品の研究・開発・実証補助金 2022年度 水素関連製品の研究・開発・実証補助金</t>
@@ -2619,8 +2569,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>神戸市では、ビジネス環境の変化への対応が求められる市内中小企業のDX推進を支援するため、デジタル技術を活用した経営課題の解決や事業転換を行う事業者を対象とする補助制度を実施します。 2025年度 神戸市中小企業DX推進支援補助制度 （参考） 2024年度 神戸市中小企業DX推進支援補助制度</t>
@@ -2653,8 +2601,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>神戸市では、戦略産業分野に関する独自で選定したテーマに取り組む市内中小企業を中心とした企業グループに対し補助金を交付することで、神戸挑戦企業等支援補助制度の目的である市内中小企業のものづくり技術の高度化及び市内産業の振興を図るとともに、意欲ある市内企業の成長を促すことを目的としています。 2025年度「中小企業チャレンジサポート補助金」公募について 【参考】 2024年度「中小企業チャレンジサポート補助金」公募について 2023年度「…</t>
@@ -2687,7 +2633,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>上限額：2,000万円</t>
@@ -2725,7 +2670,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>250万円</t>
@@ -2763,7 +2707,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>150万円</t>
@@ -2806,7 +2749,6 @@
           <t>2023-05-30</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>本市では2023年度、戦略産業分野（「航空・宇宙」「医療・健康・福祉」「農業・食糧」「環境・エネルギー（水素除く）」）における新事業展開のための試作開発や新素材・新製品の実用化に向けた開発、大学・公設試等の研究機関等と連携し社会課題の解決につながる革新的な開発に取り組む、神戸市内中小企業若しくは神戸市内中小企業等により構成されるコンソーシアムに対し、補助金交付等を支援する「神戸挑戦企業等支援補助制度」を実施します。 また、2023年度…</t>
@@ -2844,7 +2786,6 @@
           <t>2024-05-20</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>本市では2024年度、戦略産業分野（「航空・宇宙」「医療・健康・福祉」「農業・食糧」「環境・エネルギー（水素除く）」）における新事業展開のための試作開発や新素材・新製品の実用化に向けた開発、大学・公設試等の研究機関等と連携し社会課題の解決につながる革新的な開発に取り組む、神戸市内中小企業若しくは神戸市内中小企業等により構成されるコンソーシアムを、補助金交付等により支援する「神戸挑戦企業等支援補助制度」を実施します。 また、「カーボンニ…</t>
@@ -2877,7 +2818,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>150万円</t>
@@ -2915,7 +2855,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>上限150万円</t>
@@ -2953,7 +2892,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>150万円</t>
@@ -2991,8 +2929,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>神戸市では、人手不足や物価高騰等の社会課題への対応と市内産業の振興を図るため、幅広い業種や事業の業務の省力化につながる製品を開発する市内企業等に対して、その研究・開発・実証にかかる費用を補助します。 2026年度「省力化を促進する製品の研究・開発・実証補助金」 【参考】 2025年度「省力化を促進する製品の研究・開発・実証補助金」 2026年度「省力化を促進する製品の研究・開発・実証補助金」</t>
@@ -3030,7 +2966,6 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>ファッション産業分野において、産業固有の課題解決や地域ブランドのブランド力向上を目的に行われる普及啓発活動や販売促進活動、新たな製品の開発又は改良等に関する経費を支援し、神戸ブランドのさらなる魅力向上を図ります。 募集の案内 定義 ファッション産業 神戸の歴史、自然及び文化を生かし、並びに地域に根差した地場産業等ファッション性豊かな衣・食・住・遊にわたる生活文化産業全般をいいます。 中小企業 中小企業基本法（昭和38年法律第154号）…</t>
@@ -3063,7 +2998,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>4,000円</t>
@@ -3143,7 +3077,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>上限100万円</t>
@@ -3181,7 +3114,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
           <t>4,000円</t>
@@ -3219,7 +3151,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
           <t>上限 補助限度額 100万円</t>
@@ -3341,8 +3272,6 @@
           <t>公募中</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>西宮市の起業家・事業者むけ支援メニュー【セミナー・補助金など】 更新日：2025年10月29日 ページ番号：76218586 当ページでは、西宮市の起業家および事業者への各種支援メニューをご案内します。 目次 相談先のご案内 セミナーのご案内 特定創業支援等事業のご案内 補助金のご案内 専門家派遣のご案内 役立つホームページのご案内 事業承継のご相談 1．相談先のご案内 A にしのみや起業家支援センター みやスタ にしのみや起業家支援…</t>
@@ -3380,7 +3309,6 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>本サイトでは 創業型第1回公募以降 の情報を掲載しています。 そのほかすべての型の公募情報は、 小規模事業者持続化補助金まとめサイト にてご確認ください。 小規模事業者持続化補助金＜創業型＞の申請要件 ※第3回から変更となりました。 産業競争力強化法に基づく「認定市区町村」または「認定市区町村」と連携した「認定連携創業支援等事業者」が実施した「特定創業支援等事業」による支援を受けた日および開業日（設立年月日）が下記期間内であること。 …</t>
@@ -3418,7 +3346,6 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>本サイトでは 第17回公募以降 の情報を掲載しています。 過去回およびすべての型の公募情報は、 小規模事業者持続化補助金まとめサイト にてご確認ください。 今後のスケジュール 次回公募については、詳細の公開までお待ちください。 予定は変更する場合があります。スケジュールの詳細は こちら をご確認ください。 これから応募される方はこちら （応募ページへ） 採択された方はこちら （採択後の流れへ） －各種動画一覧－ ※外部サイトが開きます…</t>
@@ -3451,8 +3378,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>IT導入補助金（外部サイト）</t>
@@ -3490,7 +3415,6 @@
           <t>2025-04-22</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>NEWS すべて HP更新 イベント 2025.06.26 ご案内 補助事業により取得した資産についてのご注意 2024.10.08 ご案内 事業化状況報告未提出による交付決定取消事案発生のお知らせ 事業化状況報告に関する注意喚起について 2026.04.03 HP更新 「Jグランツ事業者マニュアル」を更新しました。 2026.03.30 HP更新 「補助事業の手引き」を更新しました。 2026.03.27 ご案内 補助事業者に対する…</t>
@@ -3523,7 +3447,6 @@
           <t>公募中</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>最大1500万円</t>
@@ -3561,7 +3484,6 @@
           <t>公募開始</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>1,000円</t>
@@ -3641,7 +3563,6 @@
           <t>公募予定</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>限度額 補助率 留意点 工事費 新規出店に伴う店舗部分の内装及び外装の工事費 50万円</t>
@@ -3679,7 +3600,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>限度額 50万円</t>
@@ -3717,7 +3637,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>限度額 20万円</t>
@@ -3755,7 +3674,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>限度額 50万円</t>
@@ -3774,6 +3692,86 @@
       <c r="H87" t="inlineStr">
         <is>
           <t>2026-05-04 02:16:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>西宮市子ども食堂運営支援事業補助金について</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>上限は年度で52万円</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>更新日：2026年3月19日 ページ番号：27004411 市内の子ども食堂に対する支援として、西宮市子ども食堂運営支援事業補助金事業について募集します。 西宮市子ども食堂運営支援事業補助金 概要 西宮市では、地域との交流、学習支援及び地域の子供の居場所づくりを促進するため、子ども食堂が実施する以下の2つの事業（以下「事業」という。）に要する経費の一部を補助します。 食事を提供する事業 地域との交流、学習支援及び子供の居場所づくり事業…</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kenko/shakaifukushi/chiikifukushi/kodomoshokudo.html</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:10:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>西宮市青少年地域活性化支援事業補助金のご案内</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>5万円</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>更新日：2026年3月28日 ページ番号：70246178 （制度）概要 青少年が実施するコミュニティ活動を支援 市は、地域に根ざした活動を行っている青少年層により組織された団体が実施する地域への貢献や活性化に寄与する事業に対し、西宮市青少年地域活性化支援事業補助金を交付します。 この補助金を交付することにより、地域コミュニティの次世代の担い手を育成し、地域コミュニティ活動の推進及び地域の活性化を図ることを目的としています。 対象者・…</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/shisei/sankaku/community/josei/seishonen-hojokin.html</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:10:49</t>
         </is>
       </c>
     </row>
@@ -3859,8 +3857,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>神戸市では、市内中小企業の操業基盤の強化を図るため、技術力や生産性の向上、受注拡大、研究開発機能の強化などに向けた設備投資等を行う事業者を対象とする助成制度を実施しています。 2026年度 神戸市中小企業投資促進等助成制度 【参考】 2025年度 神戸市中小企業投資促進等助成制度 2024年度 神戸市中小企業投資促進等助成制度 2023年度 神戸市中小企業投資促進等助成制度 2022年度(令和4年度) 神戸市中小製造業投資促進等助成制…</t>
@@ -3893,8 +3889,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>神戸市では、戦略産業分野における新事業展開のための試作開発や新素材・新製品の実用化に向けた開発、大学・公設試等の研究機関等と連携し社会課題の解決につながる革新的な開発に取り組む神戸市内中小企業若しくは神戸市内中小企業等により構成されるコンソーシアムに対し補助金を交付することにより、ものづくり技術の高度化と市内産業の振興を図ることを目的としています。 2025年度「神戸挑戦企業等支援補助制度」 （参考） 2024年度「神戸挑戦企業等支援…</t>
@@ -3927,8 +3921,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>神戸市では、水素関連製品の実用化に向けた研究・開発・実証に取り組む、神戸市内の中小企業若しくは神戸市内の中小企業等より構成されるコンソーシアムを対象とする補助制度を実施しています。 2025年度 水素関連製品の研究・開発・実証補助金 （参考） 2024年度 水素関連製品の研究・開発・実証補助金 2023年度 水素関連製品の研究・開発・実証補助金 2022年度 水素関連製品の研究・開発・実証補助金</t>
@@ -3961,8 +3953,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>神戸市では、ビジネス環境の変化への対応が求められる市内中小企業のDX推進を支援するため、デジタル技術を活用した経営課題の解決や事業転換を行う事業者を対象とする補助制度を実施します。 2025年度 神戸市中小企業DX推進支援補助制度 （参考） 2024年度 神戸市中小企業DX推進支援補助制度</t>
@@ -3995,8 +3985,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>神戸市では、戦略産業分野に関する独自で選定したテーマに取り組む市内中小企業を中心とした企業グループに対し補助金を交付することで、神戸挑戦企業等支援補助制度の目的である市内中小企業のものづくり技術の高度化及び市内産業の振興を図るとともに、意欲ある市内企業の成長を促すことを目的としています。 2025年度「中小企業チャレンジサポート補助金」公募について 【参考】 2024年度「中小企業チャレンジサポート補助金」公募について 2023年度「…</t>
@@ -4029,7 +4017,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>上限額：2,000万円</t>
@@ -4067,7 +4054,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>250万円</t>
@@ -4105,7 +4091,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>150万円</t>
@@ -4148,7 +4133,6 @@
           <t>2023-05-30</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>本市では2023年度、戦略産業分野（「航空・宇宙」「医療・健康・福祉」「農業・食糧」「環境・エネルギー（水素除く）」）における新事業展開のための試作開発や新素材・新製品の実用化に向けた開発、大学・公設試等の研究機関等と連携し社会課題の解決につながる革新的な開発に取り組む、神戸市内中小企業若しくは神戸市内中小企業等により構成されるコンソーシアムに対し、補助金交付等を支援する「神戸挑戦企業等支援補助制度」を実施します。 また、2023年度…</t>
@@ -4186,7 +4170,6 @@
           <t>2024-05-20</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>本市では2024年度、戦略産業分野（「航空・宇宙」「医療・健康・福祉」「農業・食糧」「環境・エネルギー（水素除く）」）における新事業展開のための試作開発や新素材・新製品の実用化に向けた開発、大学・公設試等の研究機関等と連携し社会課題の解決につながる革新的な開発に取り組む、神戸市内中小企業若しくは神戸市内中小企業等により構成されるコンソーシアムを、補助金交付等により支援する「神戸挑戦企業等支援補助制度」を実施します。 また、「カーボンニ…</t>
@@ -4219,7 +4202,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>150万円</t>
@@ -4257,7 +4239,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>上限150万円</t>
@@ -4295,7 +4276,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>150万円</t>
@@ -4333,8 +4313,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>神戸市では、人手不足や物価高騰等の社会課題への対応と市内産業の振興を図るため、幅広い業種や事業の業務の省力化につながる製品を開発する市内企業等に対して、その研究・開発・実証にかかる費用を補助します。 2026年度「省力化を促進する製品の研究・開発・実証補助金」 【参考】 2025年度「省力化を促進する製品の研究・開発・実証補助金」 2026年度「省力化を促進する製品の研究・開発・実証補助金」</t>
@@ -4372,7 +4350,6 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>ファッション産業分野において、産業固有の課題解決や地域ブランドのブランド力向上を目的に行われる普及啓発活動や販売促進活動、新たな製品の開発又は改良等に関する経費を支援し、神戸ブランドのさらなる魅力向上を図ります。 募集の案内 定義 ファッション産業 神戸の歴史、自然及び文化を生かし、並びに地域に根差した地場産業等ファッション性豊かな衣・食・住・遊にわたる生活文化産業全般をいいます。 中小企業 中小企業基本法（昭和38年法律第154号）…</t>
@@ -4471,7 +4448,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>4,000円</t>
@@ -4551,7 +4527,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>上限100万円</t>
@@ -4589,7 +4564,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>4,000円</t>
@@ -4627,7 +4601,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>上限 補助限度額 100万円</t>
@@ -4810,7 +4783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4881,8 +4854,6 @@
           <t>公募中</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>西宮市の起業家・事業者むけ支援メニュー【セミナー・補助金など】 更新日：2025年10月29日 ページ番号：76218586 当ページでは、西宮市の起業家および事業者への各種支援メニューをご案内します。 目次 相談先のご案内 セミナーのご案内 特定創業支援等事業のご案内 補助金のご案内 専門家派遣のご案内 役立つホームページのご案内 事業承継のご相談 1．相談先のご案内 A にしのみや起業家支援センター みやスタ にしのみや起業家支援…</t>
@@ -4920,7 +4891,6 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>本サイトでは 創業型第1回公募以降 の情報を掲載しています。 そのほかすべての型の公募情報は、 小規模事業者持続化補助金まとめサイト にてご確認ください。 小規模事業者持続化補助金＜創業型＞の申請要件 ※第3回から変更となりました。 産業競争力強化法に基づく「認定市区町村」または「認定市区町村」と連携した「認定連携創業支援等事業者」が実施した「特定創業支援等事業」による支援を受けた日および開業日（設立年月日）が下記期間内であること。 …</t>
@@ -4958,7 +4928,6 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>本サイトでは 第17回公募以降 の情報を掲載しています。 過去回およびすべての型の公募情報は、 小規模事業者持続化補助金まとめサイト にてご確認ください。 今後のスケジュール 次回公募については、詳細の公開までお待ちください。 予定は変更する場合があります。スケジュールの詳細は こちら をご確認ください。 これから応募される方はこちら （応募ページへ） 採択された方はこちら （採択後の流れへ） －各種動画一覧－ ※外部サイトが開きます…</t>
@@ -4991,8 +4960,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>IT導入補助金（外部サイト）</t>
@@ -5030,7 +4997,6 @@
           <t>2025-04-22</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>NEWS すべて HP更新 イベント 2025.06.26 ご案内 補助事業により取得した資産についてのご注意 2024.10.08 ご案内 事業化状況報告未提出による交付決定取消事案発生のお知らせ 事業化状況報告に関する注意喚起について 2026.04.03 HP更新 「Jグランツ事業者マニュアル」を更新しました。 2026.03.30 HP更新 「補助事業の手引き」を更新しました。 2026.03.27 ご案内 補助事業者に対する…</t>
@@ -5063,7 +5029,6 @@
           <t>公募中</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>最大1500万円</t>
@@ -5082,6 +5047,86 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-05-04 02:15:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>西宮市子ども食堂運営支援事業補助金について</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>上限は年度で52万円</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>更新日：2026年3月19日 ページ番号：27004411 市内の子ども食堂に対する支援として、西宮市子ども食堂運営支援事業補助金事業について募集します。 西宮市子ども食堂運営支援事業補助金 概要 西宮市では、地域との交流、学習支援及び地域の子供の居場所づくりを促進するため、子ども食堂が実施する以下の2つの事業（以下「事業」という。）に要する経費の一部を補助します。 食事を提供する事業 地域との交流、学習支援及び子供の居場所づくり事業…</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kenko/shakaifukushi/chiikifukushi/kodomoshokudo.html</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:10:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>西宮市青少年地域活性化支援事業補助金のご案内</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5万円</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>更新日：2026年3月28日 ページ番号：70246178 （制度）概要 青少年が実施するコミュニティ活動を支援 市は、地域に根ざした活動を行っている青少年層により組織された団体が実施する地域への貢献や活性化に寄与する事業に対し、西宮市青少年地域活性化支援事業補助金を交付します。 この補助金を交付することにより、地域コミュニティの次世代の担い手を育成し、地域コミュニティ活動の推進及び地域の活性化を図ることを目的としています。 対象者・…</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/shisei/sankaku/community/josei/seishonen-hojokin.html</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:10:49</t>
         </is>
       </c>
     </row>
@@ -5167,7 +5212,6 @@
           <t>公募開始</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>1,000円</t>
@@ -5247,7 +5291,6 @@
           <t>公募予定</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>限度額 補助率 留意点 工事費 新規出店に伴う店舗部分の内装及び外装の工事費 50万円</t>
@@ -5285,7 +5328,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>限度額 50万円</t>
@@ -5323,7 +5365,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>限度額 20万円</t>
@@ -5361,7 +5402,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>限度額 50万円</t>
@@ -5465,8 +5505,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>大阪府副業・兼業人材活用促進補助金</t>
@@ -5696,7 +5734,6 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>開催概要 大阪市は、脱炭素社会「ゼロカーボン おおさか」の実現に向けた取組を進めています。このたび、連携協定を締結している三井住友海上火災保険株式会社と株式会社バイウィルとともに、脱炭素をテーマとしたセミナー「知れば得する！脱炭素経営×補助金活用 企業が未来を創るセミナー」を開催します。本セミナーでは、脱炭素に関する最新の動向や、本市の支援策、企業における実践例など、今後の脱炭素経営に役立つ情報をご提供します。 1 日時 令和8年2月…</t>
@@ -5795,7 +5832,6 @@
           <t>公募開始</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>上限300万円</t>
@@ -5833,7 +5869,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>500万円</t>
@@ -5871,7 +5906,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>限度額300万円</t>
@@ -5909,7 +5943,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>限度額10万円</t>
@@ -5947,7 +5980,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>限度額とします。 補助限度額：300万円</t>
@@ -6027,8 +6059,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>東大阪市 東大阪市障害者雇用奨励金 ▶東大阪市障害者雇用奨励金 （別ウインドウで開く） 市内在住の障害者を市内の事業所において常用雇用労働者として雇用する事業主の方に対し、障害者の雇用促進を目的として、障害者雇用奨励金を支給しています。 問合せ先：労働雇用政策室(06-4309-3178) 東大阪市トライアル雇用支援金 ▶東大阪市トライアル雇用支援金 （別ウインドウで開く） 若年者等の雇用を促進するため、国(ハローワーク)のトライアル…</t>
@@ -6061,8 +6091,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>東大阪市では、市内中小企業者又は市内中小企業者2社以上が共同して行う 新たな技術の研究や新製品の開発に向けた取り組み 及び市内中小企業を中心に構成する企業グループが行う 経営力の向上に資する調査研究や講習会 の開催に対して助成金を交付いたします。 備考：助成金の交付にあたっては、事業計画等をご提案いただき審査会の採択を受ける必要がございます。 当助成金の詳しい内容は 公益財団法人東大阪市産業創造勤労者支援機構 (別のサイトへ移動します…</t>
@@ -6095,8 +6123,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>東大阪市では、市内製造業の新技術・新製品に関する特許権の「保護」及び「権利化」を促進させるため、出願審査請求に直接必要となる経費に対して補助金を交付しています。 当補助金の詳しい内容は 公益財団法人東大阪市産業創造勤労者支援機構(別のサイトへ移動します) をご覧ください。</t>
@@ -6195,8 +6221,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>ページ番号1018028 補助金・融資・相談等 企業支援・産業振興に関するイベント・セミナー 産業振興のための施策 市内商工業や商店街イベントについての情報発信 吹田市ふるさと納税 工場立地・小売店舗出店に係る届け出 このページに関する お問い合わせ 都市魅力部 地域経済振興室 〒564-8550 大阪府吹田市泉町1丁目3番40号（低層棟3階316番窓口、高層棟7階706番窓口） 電話番号： 【庶務】 06-6384-1356 【企業…</t>
@@ -6229,8 +6253,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>ページ番号1018029 起業・創業 事業者向けの補助金 商店街向けの補助金 税制優遇制度 中小企業向けの融資制度 事業承継支援 相談制度 ご意見をお聞かせください このページに問題点はありましたか？（複数回答可） 特にない 内容が分かりにくい ページを探しにくい 情報が少ない 文章量が多い 送信</t>
@@ -6305,7 +6327,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>上限） 20万円</t>
@@ -6511,7 +6532,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>上限額500万円</t>
@@ -6549,7 +6569,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>上限額500万円</t>
@@ -6629,8 +6648,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>ページ番号1018058 地元企業等共同研究開発事業補助金の直近5年分の交付実績を公開しています。 令和6年度 地元企業等共同研究開発事業補助金 交付実績 令和5年度 地元企業等共同研究開発事業補助金 交付実績 令和4年度 地元企業等共同研究開発事業補助金 交付実績 令和3年度 地元企業等共同研究開発事業補助金 交付実績 令和2年度 地元企業等共同研究開発事業補助金 交付実績 このページに関する お問い合わせ 都市魅力部 地域経済振興…</t>
@@ -6663,8 +6680,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>ページ番号1021242 商店街活性化のための補助 商店街等の空き店舗活用事業 ご意見をお聞かせください このページに問題点はありましたか？（複数回答可） 特にない 内容が分かりにくい ページを探しにくい 情報が少ない 文章量が多い 送信</t>
@@ -6763,7 +6778,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>上限300万円</t>
@@ -6801,7 +6815,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>補助上限が20万円</t>
@@ -6839,7 +6852,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>限度額15万円</t>
@@ -7003,7 +7015,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>上限10万円</t>
@@ -7083,7 +7094,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>補助上限額：30万円</t>
@@ -7121,7 +7131,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>補助上限額：10万円</t>
@@ -7159,7 +7168,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>補助上限： 10万円</t>
@@ -7323,7 +7331,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>上限】1億円</t>
@@ -7361,7 +7368,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>上限 300万円</t>
@@ -7399,7 +7405,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>上限 500万円</t>
@@ -7437,7 +7442,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>上限 250万円</t>
@@ -7475,8 +7479,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>令和6年度豊中市チャレンジ事業補助金の申込受付は終了しました</t>
@@ -7575,7 +7577,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>上限額：30万円</t>
@@ -7721,8 +7722,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>本文 建築物の耐震化（補助金等） お知らせ 2026年4月1日更新 耐震診断・改修事業者情報提供制度 制度・事業等 2026年4月1日更新 木造住宅耐震事業費用の補助制度 2026年4月1日更新 木造住宅除却工事補助制度補助 2023年3月31日更新 分譲マンションの耐震補助制度 2023年3月31日更新 （木造以外）耐震診断費用の補助制度 手続き 2022年3月30日更新 耐震事業者のみなさまへ 計画 2026年4月1日更新 高槻市…</t>
@@ -7755,8 +7754,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>本文 ブロック塀等の安全確保（補助金等） お知らせ 2026年4月1日更新 ブロック塀撤去事業者の情報提供 2022年3月22日更新 塀の安全点検 制度・事業等 2025年4月1日更新 ブロック塀等撤去工事費の補助制度 2022年3月22日更新 高槻市ブロック塀等の安全確保に向けた手引き</t>
@@ -7855,7 +7852,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>15,000,000円</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-05-08 14:52 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="尼崎市" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="西宮市" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="川西市" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="堺市" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3711,7 +3712,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>上限は年度で52万円</t>
@@ -3772,6 +3772,44 @@
       <c r="H89" t="inlineStr">
         <is>
           <t>2026-05-07 17:10:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>堺市子育て世帯等空き家活用定住支援事業補助金</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月30日 お知らせ 令和8年度の堺市子育て世帯等空き家活用定住支援事業を行います。 申請受付は令和8年5月1日から令和9年1月29日までです。 ・ 空き家 は既存住宅（ 居住用に使用されたことのある住宅 ）が対象です。 ・ 令和7年4月1日以降 の空き家の購入者が対象です。 ・ 令和8年2月28日 から 令和9年1月29日 に空き家の住所に住民票を 異動 した世帯が対象です。 ※ 【フラット35】（地域連携型） が…</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/jutaku/jutaku/akiya_rikatsuyou/teiju_hojo.html</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:48:57</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5104,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>上限は年度で52万円</t>
@@ -5428,6 +5465,110 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>自治体名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>補助金名</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>公募ステータス</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>締切日</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>補助金額(上限)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>概要</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>取得日時</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>堺市子育て世帯等空き家活用定住支援事業補助金</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月30日 お知らせ 令和8年度の堺市子育て世帯等空き家活用定住支援事業を行います。 申請受付は令和8年5月1日から令和9年1月29日までです。 ・ 空き家 は既存住宅（ 居住用に使用されたことのある住宅 ）が対象です。 ・ 令和7年4月1日以降 の空き家の購入者が対象です。 ・ 令和8年2月28日 から 令和9年1月29日 に空き家の住所に住民票を 異動 した世帯が対象です。 ※ 【フラット35】（地域連携型） が…</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/jutaku/jutaku/akiya_rikatsuyou/teiju_hojo.html</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:48:57</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-05-14 17:17 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3796,7 +3796,6 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>更新日：2026年4月30日 お知らせ 令和8年度の堺市子育て世帯等空き家活用定住支援事業を行います。 申請受付は令和8年5月1日から令和9年1月29日までです。 ・ 空き家 は既存住宅（ 居住用に使用されたことのある住宅 ）が対象です。 ・ 令和7年4月1日以降 の空き家の購入者が対象です。 ・ 令和8年2月28日 から 令和9年1月29日 に空き家の住所に住民票を 異動 した世帯が対象です。 ※ 【フラット35】（地域連携型） が…</t>
@@ -3810,6 +3809,40 @@
       <c r="H90" t="inlineStr">
         <is>
           <t>2026-05-08 14:48:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>中小企業WEBデザイン活用事業補助金に係る登録作成事業者</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>ページ番号1044083 更新日 2026年5月14日 中小企業WEBデザイン活用事業補助金登録作成事業者 令和8年度登録作成事業者一覧 No 事業者名 ホームページ作成・改修 動画作成 SNSブランディング事業 電話番号 1 target_blank （外部リンク） 概要書 （PDF 232.8 KB） 090-6870-3869 2 クラウズカンパニー （外部リンク） 概要書 （PDF 137.0 KB） 概要書 （PDF 132…</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://www.city.suita.osaka.jp/sangyo/1018028/1018029/1018030/1044083.html</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>2026-05-14 17:14:54</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5580,6 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>更新日：2026年4月30日 お知らせ 令和8年度の堺市子育て世帯等空き家活用定住支援事業を行います。 申請受付は令和8年5月1日から令和9年1月29日までです。 ・ 空き家 は既存住宅（ 居住用に使用されたことのある住宅 ）が対象です。 ・ 令和7年4月1日以降 の空き家の購入者が対象です。 ・ 令和8年2月28日 から 令和9年1月29日 に空き家の住所に住民票を 異動 した世帯が対象です。 ※ 【フラット35】（地域連携型） が…</t>
@@ -6291,7 +6323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6834,6 +6866,40 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>2026-05-04 02:14:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>中小企業WEBデザイン活用事業補助金に係る登録作成事業者</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ページ番号1044083 更新日 2026年5月14日 中小企業WEBデザイン活用事業補助金登録作成事業者 令和8年度登録作成事業者一覧 No 事業者名 ホームページ作成・改修 動画作成 SNSブランディング事業 電話番号 1 target_blank （外部リンク） 概要書 （PDF 232.8 KB） 090-6870-3869 2 クラウズカンパニー （外部リンク） 概要書 （PDF 137.0 KB） 概要書 （PDF 132…</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.city.suita.osaka.jp/sangyo/1018028/1018029/1018030/1044083.html</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-05-14 17:14:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-05-15 17:35 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3828,8 +3828,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>ページ番号1044083 更新日 2026年5月14日 中小企業WEBデザイン活用事業補助金登録作成事業者 令和8年度登録作成事業者一覧 No 事業者名 ホームページ作成・改修 動画作成 SNSブランディング事業 電話番号 1 target_blank （外部リンク） 概要書 （PDF 232.8 KB） 090-6870-3869 2 クラウズカンパニー （外部リンク） 概要書 （PDF 137.0 KB） 概要書 （PDF 132…</t>
@@ -3843,6 +3841,48 @@
       <c r="H91" t="inlineStr">
         <is>
           <t>2026-05-14 17:14:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>令和8年度堺市中小企業デジタル化促進補助金</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>100万円</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月15日 事業概要 人手不足や原油価格高騰をはじめとする、企業を取り巻く環境が急激に変化している中、市内中小企業の生産性向上をめざし、市内中小企業がデジタルツールを活用して、将来にわたり継続的に自社の業務の成長・発展に取り組む費用の一部を補助します。 補助金に関する詳細は、以下の募集要領に記載していますので、申請をご検討の際は必ずご覧ください。 また、申請に際しては、堺市産業振興センターの「産業DX支援センター」又…</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/dx_shien/digitalka.html</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:32:45</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5593,6 +5633,48 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-05-08 14:48:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>令和8年度堺市中小企業デジタル化促進補助金</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>100万円</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月15日 事業概要 人手不足や原油価格高騰をはじめとする、企業を取り巻く環境が急激に変化している中、市内中小企業の生産性向上をめざし、市内中小企業がデジタルツールを活用して、将来にわたり継続的に自社の業務の成長・発展に取り組む費用の一部を補助します。 補助金に関する詳細は、以下の募集要領に記載していますので、申請をご検討の際は必ずご覧ください。 また、申請に際しては、堺市産業振興センターの「産業DX支援センター」又…</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/dx_shien/digitalka.html</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:32:45</t>
         </is>
       </c>
     </row>
@@ -6885,8 +6967,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>ページ番号1044083 更新日 2026年5月14日 中小企業WEBデザイン活用事業補助金登録作成事業者 令和8年度登録作成事業者一覧 No 事業者名 ホームページ作成・改修 動画作成 SNSブランディング事業 電話番号 1 target_blank （外部リンク） 概要書 （PDF 232.8 KB） 090-6870-3869 2 クラウズカンパニー （外部リンク） 概要書 （PDF 137.0 KB） 概要書 （PDF 132…</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-05-18 21:00 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3883,6 +3883,48 @@
       <c r="H92" t="inlineStr">
         <is>
           <t>2026-05-15 17:32:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>高槻市</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>令和8年度　高槻市配食サービス事業者物価高対策支援金</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>15万円</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>本文 令和8年度 高槻市配食サービス事業者物価高対策支援金 ページID：165819 更新日：2026年5月18日更新 印刷ページ表示 令和8年度 高槻市配食サービス事業者物価高対策支援金 物価高の影響により、調理が困難な高齢者や重度の障がい者の栄養改善と安否確認を目的として実施している、高槻市に本社をおく配食サービス事業者に対して支援金を交付します。 対象となる事業 高槻市に在住する、調理が困難な高齢者または、重度の障がい者に対して…</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.city.takatsuki.osaka.jp/soshiki/35/165819.html</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2026-05-18 20:59:23</t>
         </is>
       </c>
     </row>
@@ -7938,7 +7980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8054,6 +8096,48 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>2026-05-04 02:14:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>高槻市</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>令和8年度　高槻市配食サービス事業者物価高対策支援金</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>15万円</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>本文 令和8年度 高槻市配食サービス事業者物価高対策支援金 ページID：165819 更新日：2026年5月18日更新 印刷ページ表示 令和8年度 高槻市配食サービス事業者物価高対策支援金 物価高の影響により、調理が困難な高齢者や重度の障がい者の栄養改善と安否確認を目的として実施している、高槻市に本社をおく配食サービス事業者に対して支援金を交付します。 対象となる事業 高槻市に在住する、調理が困難な高齢者または、重度の障がい者に対して…</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.city.takatsuki.osaka.jp/soshiki/35/165819.html</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-05-18 20:59:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-05-19 19:52 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3925,6 +3925,90 @@
       <c r="H93" t="inlineStr">
         <is>
           <t>2026-05-18 20:59:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>国内展示会出展支援助成金</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【募集期間内】 交付決定通知書を受領 実績報</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>上限 10 万円</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>事業目的 国内への販路開拓を応援 市内中小企業者や中小企業者2社以上で構成される共同グループが行う、 国内展示会の出展 に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 競争力があると考えられる製品・技術を有する企業等の国内での販路開拓の支援を通じて、 本市の産業振興を図るものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支援機構ホームページ)よりご覧ください。 事業概要 市内…</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043092.html</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>2026-05-19 19:49:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>高付加価値化促進事業助成金(研究開発事業)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>提案書類を提出 【募集期間内・年3回程度】 審査会にて、 事</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>上限 50万円</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>事業目的 新技術の研究・新製品の開発を応援 市内中小企業者又は市内中小企業者2社以上が共同で行う、新技術の研究や新製品の開発に向けた取り組みに対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 付加価値の高い製品の開発や技術研究を促進するものです。(東大阪市補助事業) 詳しくは、こちら((公財) 東大阪市産業創造勤労者支援機構ホームページ)よりご覧ください。 事業概要 下記のいずれかに該当する事業のうち、事業に…</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043090.html</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-05-19 19:49:05</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6433,6 +6517,90 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-05-04 02:13:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>国内展示会出展支援助成金</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【募集期間内】 交付決定通知書を受領 実績報</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>上限 10 万円</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>事業目的 国内への販路開拓を応援 市内中小企業者や中小企業者2社以上で構成される共同グループが行う、 国内展示会の出展 に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 競争力があると考えられる製品・技術を有する企業等の国内での販路開拓の支援を通じて、 本市の産業振興を図るものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支援機構ホームページ)よりご覧ください。 事業概要 市内…</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043092.html</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-19 19:49:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>高付加価値化促進事業助成金(研究開発事業)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>提案書類を提出 【募集期間内・年3回程度】 審査会にて、 事</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>上限 50万円</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>事業目的 新技術の研究・新製品の開発を応援 市内中小企業者又は市内中小企業者2社以上が共同で行う、新技術の研究や新製品の開発に向けた取り組みに対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 付加価値の高い製品の開発や技術研究を促進するものです。(東大阪市補助事業) 詳しくは、こちら((公財) 東大阪市産業創造勤労者支援機構ホームページ)よりご覧ください。 事業概要 下記のいずれかに該当する事業のうち、事業に…</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043090.html</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-05-19 19:49:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-05-22 19:33 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4009,6 +4009,208 @@
       <c r="H95" t="inlineStr">
         <is>
           <t>2026-05-19 19:49:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>産業財産権活用事業助成金</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【随時受付】 交付決定書を受領 実績報告書を</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>上限 10 万円</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>事業目的 特許取得を応援 特許法に規定されている特許権の国内での取得費用に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 市内製造業の開発した新技術・新製品に関する産業財産権の保護及び権利化を促進し、 市内製造業の競争力強化及び事業活動の振興を目的とするものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支援機構ホームページ)よりご覧ください。 事業概要 市内製造事業者が特許出願…</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043109.html</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>海外展示会出展支援助成金</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【募集期間内】 交付決定通知書を受領 実績報</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>上限 100 万円</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>夏頃の募集開始を予定 しています。お問合せは、下記のいずれかへお願いします。 ●(公財)東大阪市産業創造勤労者支援機構 電話：06－4309－2301 ●東大阪市 都市魅力産業スポーツ部 モノづくり支援室 電話：06－4309－3177 本補助金をご検討の企業様 必見！！ 令和8年5月29日金曜日今から始める中小企業のための「海外販路開拓セミナー」を実施します。 下記チラシの二次元コードからお申し込みください。 【チラシ】0529海外…</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000044213.html</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>常設展示場出展料助成金</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【随時受付】 交付決定通知書を受領 交付請求</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>事業目的 クリエイション・コア東大阪を活用した販路開拓を応援 (独法)中小企業基盤整備機構が整備したモノづくり拠点「クリエイション・コア東大阪」の常設展示場に 優れた技術・製品を出展展示する市内製造事業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 新たなビジネスマッチング・販路開拓を生み出し、本市の産業振興を目的とするものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支…</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043104.html</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>創業促進インキュベートルーム賃料助成金</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>インキュベートルームの賃貸契約締結後、 申請書類を提出 【随</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>事業目的 新製品・新技術の開発、新事業の創出を応援 (独法)中小企業基盤整備機構の公的賃借施設「クリエイション・コア東大阪」のインキュベートルームに入居した者のうち、 本市の工業集積等を活用して、新製品・新技術の開発や新事業の創出を図る中小企業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、本市内における創業を促すものです。(東大阪市補助事業) 詳しくは、こちら((公財) 東大阪市産業創造勤労者支援機構…</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043101.html</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>高槻市</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>「将棋のまち推進」新商品創出・販路開拓促進等補助金を募集します</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>応募期間 2次募集は、令和8年8 月19 日（水曜日）午後5</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>上限50万円</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>本文 「将棋のまち推進」新商品創出・販路開拓促進等補助金を募集します ページID：130791 更新日：2026年5月22日更新 印刷ページ表示 「将棋のまち高槻」の推進につながる新商品を創出する事業者を支援します 高槻市では、関西将棋会館開館に伴い、「将棋のまち高槻」の推進に資する中小企業者等を支援するため、将棋に関連する新商品の創出にかかる費用等を補助する制度「新商品・販路開拓等補助金」事業を実施しています。 ※補助金の交付には、…</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.city.takatsuki.osaka.jp/soshiki/58/130791.html</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:32:15</t>
         </is>
       </c>
     </row>
@@ -6142,7 +6344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6601,6 +6803,166 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>2026-05-19 19:49:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>産業財産権活用事業助成金</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【随時受付】 交付決定書を受領 実績報告書を</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>上限 10 万円</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>事業目的 特許取得を応援 特許法に規定されている特許権の国内での取得費用に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 市内製造業の開発した新技術・新製品に関する産業財産権の保護及び権利化を促進し、 市内製造業の競争力強化及び事業活動の振興を目的とするものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支援機構ホームページ)よりご覧ください。 事業概要 市内製造事業者が特許出願…</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043109.html</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>海外展示会出展支援助成金</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【募集期間内】 交付決定通知書を受領 実績報</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>上限 100 万円</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>夏頃の募集開始を予定 しています。お問合せは、下記のいずれかへお願いします。 ●(公財)東大阪市産業創造勤労者支援機構 電話：06－4309－2301 ●東大阪市 都市魅力産業スポーツ部 モノづくり支援室 電話：06－4309－3177 本補助金をご検討の企業様 必見！！ 令和8年5月29日金曜日今から始める中小企業のための「海外販路開拓セミナー」を実施します。 下記チラシの二次元コードからお申し込みください。 【チラシ】0529海外…</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000044213.html</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>常設展示場出展料助成金</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>申請書類を提出 【随時受付】 交付決定通知書を受領 交付請求</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>事業目的 クリエイション・コア東大阪を活用した販路開拓を応援 (独法)中小企業基盤整備機構が整備したモノづくり拠点「クリエイション・コア東大阪」の常設展示場に 優れた技術・製品を出展展示する市内製造事業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 新たなビジネスマッチング・販路開拓を生み出し、本市の産業振興を目的とするものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支…</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043104.html</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>東大阪市</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>創業促進インキュベートルーム賃料助成金</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>インキュベートルームの賃貸契約締結後、 申請書類を提出 【随</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>事業目的 新製品・新技術の開発、新事業の創出を応援 (独法)中小企業基盤整備機構の公的賃借施設「クリエイション・コア東大阪」のインキュベートルームに入居した者のうち、 本市の工業集積等を活用して、新製品・新技術の開発や新事業の創出を図る中小企業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、本市内における創業を促すものです。(東大阪市補助事業) 詳しくは、こちら((公財) 東大阪市産業創造勤労者支援機構…</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.city.higashiosaka.lg.jp/0000043101.html</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:30:48</t>
         </is>
       </c>
     </row>
@@ -8148,7 +8510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8306,6 +8668,48 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>2026-05-18 20:59:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>高槻市</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>「将棋のまち推進」新商品創出・販路開拓促進等補助金を募集します</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>応募期間 2次募集は、令和8年8 月19 日（水曜日）午後5</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>上限50万円</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>本文 「将棋のまち推進」新商品創出・販路開拓促進等補助金を募集します ページID：130791 更新日：2026年5月22日更新 印刷ページ表示 「将棋のまち高槻」の推進につながる新商品を創出する事業者を支援します 高槻市では、関西将棋会館開館に伴い、「将棋のまち高槻」の推進に資する中小企業者等を支援するため、将棋に関連する新商品の創出にかかる費用等を補助する制度「新商品・販路開拓等補助金」事業を実施しています。 ※補助金の交付には、…</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.city.takatsuki.osaka.jp/soshiki/58/130791.html</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-22 19:32:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-09 08:25 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4117,7 +4117,6 @@
           <t>申請書類を提出 【随時受付】 交付決定通知書を受領 交付請求</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>事業目的 クリエイション・コア東大阪を活用した販路開拓を応援 (独法)中小企業基盤整備機構が整備したモノづくり拠点「クリエイション・コア東大阪」の常設展示場に 優れた技術・製品を出展展示する市内製造事業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 新たなビジネスマッチング・販路開拓を生み出し、本市の産業振興を目的とするものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支…</t>
@@ -4155,7 +4154,6 @@
           <t>インキュベートルームの賃貸契約締結後、 申請書類を提出 【随</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>事業目的 新製品・新技術の開発、新事業の創出を応援 (独法)中小企業基盤整備機構の公的賃借施設「クリエイション・コア東大阪」のインキュベートルームに入居した者のうち、 本市の工業集積等を活用して、新製品・新技術の開発や新事業の創出を図る中小企業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、本市内における創業を促すものです。(東大阪市補助事業) 詳しくは、こちら((公財) 東大阪市産業創造勤労者支援機構…</t>
@@ -4211,6 +4209,44 @@
       <c r="H100" t="inlineStr">
         <is>
           <t>2026-05-22 19:32:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>高槻市</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>運送事業者物価高対策支援金</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>公募予定</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>10万円</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>本文 運送事業者物価高対策支援金 ページID：079278 更新日：2026年6月8日更新 印刷ページ表示 原油価格や物価の高騰により経営に影響を受けながらも、事業の継続に努める貨物運送事業者に対し、市独自の支援金を支給します。 対象者 次の1から4のすべてに該当する事業者 中小企業信用保険法第2条に規定する中小企業者（個人事業主含む） 貨物自動車運送事業法（平成元年法律第83号）に基づく一般貨物自動車運送事業、特定貨物自動車運送事業…</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.city.takatsuki.osaka.jp/soshiki/58/79278.html</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-06-09 08:24:28</t>
         </is>
       </c>
     </row>
@@ -6911,7 +6947,6 @@
           <t>申請書類を提出 【随時受付】 交付決定通知書を受領 交付請求</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>事業目的 クリエイション・コア東大阪を活用した販路開拓を応援 (独法)中小企業基盤整備機構が整備したモノづくり拠点「クリエイション・コア東大阪」の常設展示場に 優れた技術・製品を出展展示する市内製造事業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、 新たなビジネスマッチング・販路開拓を生み出し、本市の産業振興を目的とするものです。(東大阪市補助事業) 詳しくは、こちら((公財)東大阪市産業創造勤労者支…</t>
@@ -6949,7 +6984,6 @@
           <t>インキュベートルームの賃貸契約締結後、 申請書類を提出 【随</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>事業目的 新製品・新技術の開発、新事業の創出を応援 (独法)中小企業基盤整備機構の公的賃借施設「クリエイション・コア東大阪」のインキュベートルームに入居した者のうち、 本市の工業集積等を活用して、新製品・新技術の開発や新事業の創出を図る中小企業者等に対して、 (公財)東大阪市産業創造勤労者支援機構が助成金を交付することで、本市内における創業を促すものです。(東大阪市補助事業) 詳しくは、こちら((公財) 東大阪市産業創造勤労者支援機構…</t>
@@ -8510,7 +8544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8710,6 +8744,44 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>2026-05-22 19:32:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>高槻市</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>運送事業者物価高対策支援金</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>公募予定</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>10万円</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>本文 運送事業者物価高対策支援金 ページID：079278 更新日：2026年6月8日更新 印刷ページ表示 原油価格や物価の高騰により経営に影響を受けながらも、事業の継続に努める貨物運送事業者に対し、市独自の支援金を支給します。 対象者 次の1から4のすべてに該当する事業者 中小企業信用保険法第2条に規定する中小企業者（個人事業主含む） 貨物自動車運送事業法（平成元年法律第83号）に基づく一般貨物自動車運送事業、特定貨物自動車運送事業…</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.city.takatsuki.osaka.jp/soshiki/58/79278.html</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-06-09 08:24:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-16 09:02 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4228,7 +4228,6 @@
           <t>公募予定</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>10万円</t>
@@ -4247,6 +4246,48 @@
       <c r="H101" t="inlineStr">
         <is>
           <t>2026-06-09 08:24:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>創業支援型事業所賃借料補助金</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>補助上限額 5万円</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>ページ番号1023431 更新日 2026年6月15日 制度概要 趣旨 地域経済の活性化につながる創業を市内で実施する創業者に事業所賃借料の一部を補助します。 補助金の交付を受けるためには、認定会議において、創業計画のプレゼンテーションを行い、認定を受ける必要があります。 補助対象者 吹田市内で創業を計画しており、以下のいずれにも該当すること。 これまで事業を営んでいない個人であること。 認定を受けた創業計画を開始する時点において、そ…</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.city.suita.osaka.jp/sangyo/1018028/1018029/1018030/1023431.html</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:00:30</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7586,6 +7627,48 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>2026-05-14 17:14:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>創業支援型事業所賃借料補助金</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>補助上限額 5万円</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ページ番号1023431 更新日 2026年6月15日 制度概要 趣旨 地域経済の活性化につながる創業を市内で実施する創業者に事業所賃借料の一部を補助します。 補助金の交付を受けるためには、認定会議において、創業計画のプレゼンテーションを行い、認定を受ける必要があります。 補助対象者 吹田市内で創業を計画しており、以下のいずれにも該当すること。 これまで事業を営んでいない個人であること。 認定を受けた創業計画を開始する時点において、そ…</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.city.suita.osaka.jp/sangyo/1018028/1018029/1018030/1023431.html</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:00:30</t>
         </is>
       </c>
     </row>
@@ -8763,7 +8846,6 @@
           <t>公募予定</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>10万円</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-17 08:49 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4288,6 +4288,48 @@
       <c r="H102" t="inlineStr">
         <is>
           <t>2026-06-16 09:00:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>先端設備等導入支援補助金</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>300万円</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>更新日：2026年6月1日 制度の趣旨 エネルギー価格高騰の影響や人手不足等に対応するため、省力化・合理化等を図ろうとする前向きな投資を行う市内中小企業者を支援することを目的に、労働生産性を向上させる先端設備等の導入に係る経費を補助します。 本補助金は、国の「物価高騰対応重点支援地方創生臨時交付金」を原資としており、国の間接補助にあたります。国等他の補助制度と併用する予定がある場合、必ず当該補助金の事務局等に、国庫支出金を原資とする地…</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/kigyoricchi/sentanhojyo.html</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-06-17 08:46:12</t>
         </is>
       </c>
     </row>
@@ -5949,7 +5991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6080,6 +6122,48 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>2026-05-15 17:32:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>先端設備等導入支援補助金</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>300万円</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>更新日：2026年6月1日 制度の趣旨 エネルギー価格高騰の影響や人手不足等に対応するため、省力化・合理化等を図ろうとする前向きな投資を行う市内中小企業者を支援することを目的に、労働生産性を向上させる先端設備等の導入に係る経費を補助します。 本補助金は、国の「物価高騰対応重点支援地方創生臨時交付金」を原資としており、国の間接補助にあたります。国等他の補助制度と併用する予定がある場合、必ず当該補助金の事務局等に、国庫支出金を原資とする地…</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/kigyoricchi/sentanhojyo.html</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-06-17 08:46:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-20 08:16 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4330,6 +4330,170 @@
       <c r="H103" t="inlineStr">
         <is>
           <t>2026-06-17 08:46:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>堺市女性雇用促進等職場環境整備支援事業補助金のご案内</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>公募予定</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">申請関係書類 申請募集期間 対象者 補助内容 申請必要書類 </t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>上限50万円</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 堺市では、女性の雇用・就労を促進することを目的として、女性の職域拡大につながる職場環境整備に必要な経費の一部を補助いたします。 目次 クリックすると、該当の項目へとびます。 申請関係書類 申請募集期間 対象者 補助内容 申請必要書類 申請等資料 申請から補助金交付の流れ 参考資料 案内チラシや過去の活用事例、よくあるご質問をまとめています。 案内チラシ 活用事例集 Q＆A 要綱・規則 補助金交付要綱・堺市補…</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/careerweb/kigyo/diversity/shokuba-hojo.html</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:12:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>堺市オープンファクトリー推進事業補助金</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>20万円</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>更新日：2026年5月1日 伝統産業の魅力を発信することで、イメージの向上及び集客による地域経済の活性化を図るため、市内の伝統産業事業者に対し、見学者及び体験者を受け入れるための環境整備にかかる経費の一部を補助します。 補助内容について 補助対象者 市内に事業所を有している伝統産業事業者。 ※「伝統産業事業者」とは、次のいずれかの伝統産品を自ら製造する事業主をいいます。 （1）刃物 （2）注染・和晒 （3）線香 （4）昆布加工（手すき…</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/openfactoryhojyo.html</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:12:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>令和8年度 堺市新事業チャレンジ支援補助金</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>3,000千円</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 中小企業者の製品・技術・サービス等の高付加価値化や、新分野進出の円滑化等に資することを目的に、新たな事業にチャレンジする経費を補助します。詳しくは募集要領をご覧ください。 概要 期 間 1年（令和8年4月1日から令和9年3月31日まで） 上 限 3,000千円 補助率 補助対象経費の1/2 事業計画の要件 次のすべてを満たすことが必要です。 （1）申請者が主体となって実施する新製品・新技術等の開発を伴う事業…</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/chusho/proddev/monochalle.html</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:12:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>西宮市医療機関等及び介護施設等DX推進補助金</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>上限200,000円</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>更新日：2026年5月20日 ページ番号：63888886 重要 本補助金は、交付決定（7月末を予定）後に発注や購入をする経費が対象です。 交付決定前に着手したものは対象外となりますので、ご注意ください。 1．概要 今般の物価高騰が医療機関等及び介護施設等の経営を圧迫している中、限られた資源や人員の中で医療の質の維持・向上、業務の効率化等を図ることを目的に、国の「物価高騰対応重点支援地方創生臨時交付金」を活用し、西宮市独自の支援策とし…</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kenko/hokenjojoho/hokensho-news/iryoukaigodxhojokinn.html</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:15:54</t>
         </is>
       </c>
     </row>
@@ -5341,7 +5505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5684,6 +5848,48 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>2026-05-07 17:10:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>西宮市医療機関等及び介護施設等DX推進補助金</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>上限200,000円</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>更新日：2026年5月20日 ページ番号：63888886 重要 本補助金は、交付決定（7月末を予定）後に発注や購入をする経費が対象です。 交付決定前に着手したものは対象外となりますので、ご注意ください。 1．概要 今般の物価高騰が医療機関等及び介護施設等の経営を圧迫している中、限られた資源や人員の中で医療の質の維持・向上、業務の効率化等を図ることを目的に、国の「物価高騰対応重点支援地方創生臨時交付金」を活用し、西宮市独自の支援策とし…</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kenko/hokenjojoho/hokensho-news/iryoukaigodxhojokinn.html</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:15:54</t>
         </is>
       </c>
     </row>
@@ -5991,7 +6197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6164,6 +6370,128 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>2026-06-17 08:46:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>堺市女性雇用促進等職場環境整備支援事業補助金のご案内</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>公募予定</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">申請関係書類 申請募集期間 対象者 補助内容 申請必要書類 </t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>上限50万円</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 堺市では、女性の雇用・就労を促進することを目的として、女性の職域拡大につながる職場環境整備に必要な経費の一部を補助いたします。 目次 クリックすると、該当の項目へとびます。 申請関係書類 申請募集期間 対象者 補助内容 申請必要書類 申請等資料 申請から補助金交付の流れ 参考資料 案内チラシや過去の活用事例、よくあるご質問をまとめています。 案内チラシ 活用事例集 Q＆A 要綱・規則 補助金交付要綱・堺市補…</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/careerweb/kigyo/diversity/shokuba-hojo.html</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:12:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>堺市オープンファクトリー推進事業補助金</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>20万円</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>更新日：2026年5月1日 伝統産業の魅力を発信することで、イメージの向上及び集客による地域経済の活性化を図るため、市内の伝統産業事業者に対し、見学者及び体験者を受け入れるための環境整備にかかる経費の一部を補助します。 補助内容について 補助対象者 市内に事業所を有している伝統産業事業者。 ※「伝統産業事業者」とは、次のいずれかの伝統産品を自ら製造する事業主をいいます。 （1）刃物 （2）注染・和晒 （3）線香 （4）昆布加工（手すき…</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/openfactoryhojyo.html</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:12:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>令和8年度 堺市新事業チャレンジ支援補助金</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>3,000千円</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 中小企業者の製品・技術・サービス等の高付加価値化や、新分野進出の円滑化等に資することを目的に、新たな事業にチャレンジする経費を補助します。詳しくは募集要領をご覧ください。 概要 期 間 1年（令和8年4月1日から令和9年3月31日まで） 上 限 3,000千円 補助率 補助対象経費の1/2 事業計画の要件 次のすべてを満たすことが必要です。 （1）申請者が主体となって実施する新製品・新技術等の開発を伴う事業…</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/chusho/proddev/monochalle.html</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-06-20 08:12:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-23 08:45 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4391,7 +4391,6 @@
           <t>公募開始</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
           <t>20万円</t>
@@ -4494,6 +4493,44 @@
       <c r="H107" t="inlineStr">
         <is>
           <t>2026-06-20 08:15:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>設備・AI導入支援補助金</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>上限は製造業：200万円</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月24日 ページ番号：62579220 国の重点支援交付金を活用して、市内事業者に対して省力化・生産性向上設備やAIを導入する際に経費の一部を補助します 制度の概要 ・省力化・生産性向上設備導入 省力化・生産性を向上させる設備を導入する経費の一部を補助します。 補助金額は対象経費の2/3 上限は製造業：200万円、製造業以外：100万円 （補助対象経費30万円未満は対象外） 対象者は市内の中小企業・個人事業主等 ・…</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/jigyoshajoho/sangyoshinko/keieiryoku/setubiaihojo.html</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-06-23 08:45:32</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5890,6 +5927,44 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-06-20 08:15:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>設備・AI導入支援補助金</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>上限は製造業：200万円</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月24日 ページ番号：62579220 国の重点支援交付金を活用して、市内事業者に対して省力化・生産性向上設備やAIを導入する際に経費の一部を補助します 制度の概要 ・省力化・生産性向上設備導入 省力化・生産性を向上させる設備を導入する経費の一部を補助します。 補助金額は対象経費の2/3 上限は製造業：200万円、製造業以外：100万円 （補助対象経費30万円未満は対象外） 対象者は市内の中小企業・個人事業主等 ・…</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/jigyoshajoho/sangyoshinko/keieiryoku/setubiaihojo.html</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-06-23 08:45:32</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6506,6 @@
           <t>公募開始</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>20万円</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-26 08:45 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4512,7 +4512,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>上限は製造業：200万円</t>
@@ -4531,6 +4530,40 @@
       <c r="H108" t="inlineStr">
         <is>
           <t>2026-06-23 08:45:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>事業主の方のための雇用関係助成金について</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>更新日：2023年5月29日 厚生労働省が提供する助成金は、 雇用の安定、職場環境の改善、仕事と家庭の両立支援、従業員の能力向上 などに役立つものが多数あります。 詳しくは下記リンクををご参照ください。 厚生労働省「事業主の方のための雇用関係助成金」 仕事と育児・介護・治療の両立支援 助成金活用セミナー 産業振興局 産業戦略部 雇用推進課 電話番号：072-228-7404 ファクス：072-228-8816 〒590-0078 堺市…</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/careerweb/kigyo/diversity/jyoseikin.html</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:42:27</t>
         </is>
       </c>
     </row>
@@ -5946,7 +5979,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>上限は製造業：200万円</t>
@@ -6272,7 +6304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6566,6 +6598,40 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-06-20 08:12:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>事業主の方のための雇用関係助成金について</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>更新日：2023年5月29日 厚生労働省が提供する助成金は、 雇用の安定、職場環境の改善、仕事と家庭の両立支援、従業員の能力向上 などに役立つものが多数あります。 詳しくは下記リンクををご参照ください。 厚生労働省「事業主の方のための雇用関係助成金」 仕事と育児・介護・治療の両立支援 助成金活用セミナー 産業振興局 産業戦略部 雇用推進課 電話番号：072-228-7404 ファクス：072-228-8816 〒590-0078 堺市…</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/careerweb/kigyo/diversity/jyoseikin.html</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:42:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-27 08:24 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4549,8 +4549,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>更新日：2023年5月29日 厚生労働省が提供する助成金は、 雇用の安定、職場環境の改善、仕事と家庭の両立支援、従業員の能力向上 などに役立つものが多数あります。 詳しくは下記リンクををご参照ください。 厚生労働省「事業主の方のための雇用関係助成金」 仕事と育児・介護・治療の両立支援 助成金活用セミナー 産業振興局 産業戦略部 雇用推進課 電話番号：072-228-7404 ファクス：072-228-8816 〒590-0078 堺市…</t>
@@ -4564,6 +4562,82 @@
       <c r="H109" t="inlineStr">
         <is>
           <t>2026-06-26 08:42:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>大阪市</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>大阪市の脱炭素化促進に係る補助金説明会の開催について</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>大阪市は、家庭及び中小企業等の早期の省エネルギー化並びに再生可能エネルギーの導入拡大及び電力需給の安定化を図り、断熱窓及び省エネ設備等の導入加速により、大阪市の2030年度の温室効果ガス排出量削減目標達成に貢献することを目的とし補助金事業を実施します。実施にあたり、補助金の周知および円滑な活用につなげることを目的に説明会を開催します。説明会では申請にかかる注意点等をご理解いただき、申請時の不備等を減らし、事業者と行政双方の負担軽減を図…</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://www.city.osaka.lg.jp/kankyo/page/0000679117.html</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>2026-06-27 08:21:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>堺市伝統産業後継者育成事業補助金</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>5万円</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>更新日：2025年4月1日 伝統産業の後継者育成に取り組む事業主を支援することにより、後継者確保と技能の継承を図るとともに、本市の伝統産業の発展と振興に資することを目的に、新たに雇用した者に支払う賃金等を補助します。 補助対象者 市内に事業所を有している伝統産業事業主。産地組合がある場合は、当該組合に加入している者 補助対象事業 伝統産業事業主が技能を継承すべき後継者として新たに雇用し、かつ、次の全てに該当する者を育成研修する事業 伝…</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/koukeisyaikuseihojyo.html</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>2026-06-27 08:21:15</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6617,8 +6691,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>更新日：2023年5月29日 厚生労働省が提供する助成金は、 雇用の安定、職場環境の改善、仕事と家庭の両立支援、従業員の能力向上 などに役立つものが多数あります。 詳しくは下記リンクををご参照ください。 厚生労働省「事業主の方のための雇用関係助成金」 仕事と育児・介護・治療の両立支援 助成金活用セミナー 産業振興局 産業戦略部 雇用推進課 電話番号：072-228-7404 ファクス：072-228-8816 〒590-0078 堺市…</t>
@@ -6632,6 +6704,44 @@
       <c r="H8" t="inlineStr">
         <is>
           <t>2026-06-26 08:42:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>堺市伝統産業後継者育成事業補助金</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5万円</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>更新日：2025年4月1日 伝統産業の後継者育成に取り組む事業主を支援することにより、後継者確保と技能の継承を図るとともに、本市の伝統産業の発展と振興に資することを目的に、新たに雇用した者に支払う賃金等を補助します。 補助対象者 市内に事業所を有している伝統産業事業主。産地組合がある場合は、当該組合に加入している者 補助対象事業 伝統産業事業主が技能を継承すべき後継者として新たに雇用し、かつ、次の全てに該当する者を育成研修する事業 伝…</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/koukeisyaikuseihojyo.html</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-06-27 08:21:15</t>
         </is>
       </c>
     </row>
@@ -6870,7 +6980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6959,6 +7069,44 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-05-04 02:13:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>大阪市</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>大阪市の脱炭素化促進に係る補助金説明会の開催について</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>大阪市は、家庭及び中小企業等の早期の省エネルギー化並びに再生可能エネルギーの導入拡大及び電力需給の安定化を図り、断熱窓及び省エネ設備等の導入加速により、大阪市の2030年度の温室効果ガス排出量削減目標達成に貢献することを目的とし補助金事業を実施します。実施にあたり、補助金の周知および円滑な活用につなげることを目的に説明会を開催します。説明会では申請にかかる注意点等をご理解いただき、申請時の不備等を減らし、事業者と行政双方の負担軽減を図…</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.city.osaka.lg.jp/kankyo/page/0000679117.html</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-27 08:21:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-06-30 08:17 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4586,7 +4586,6 @@
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>大阪市は、家庭及び中小企業等の早期の省エネルギー化並びに再生可能エネルギーの導入拡大及び電力需給の安定化を図り、断熱窓及び省エネ設備等の導入加速により、大阪市の2030年度の温室効果ガス排出量削減目標達成に貢献することを目的とし補助金事業を実施します。実施にあたり、補助金の周知および円滑な活用につなげることを目的に説明会を開催します。説明会では申請にかかる注意点等をご理解いただき、申請時の不備等を減らし、事業者と行政双方の負担軽減を図…</t>
@@ -4619,7 +4618,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
           <t>5万円</t>
@@ -4638,6 +4636,40 @@
       <c r="H111" t="inlineStr">
         <is>
           <t>2026-06-27 08:21:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>仕事と育児・介護・治療の両立支援 助成金活用セミナー（終了しました）</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>更新日：2026年6月19日 実施内容 現在、「人口減少に伴う生産年齢人口の減少」、「仕事と育児や介護との両立など、働く方のニーズの多様化」に直面しています。こうした中、生産性の向上を図り、就業機会の拡大や意欲・能力を充分に発揮できる環境を作ることが重要な課題となっています。 本市では、働き方改革支援の観点から「両立支援等助成金（仕事と育児・介護の両立支援に取り組む事業主を応援する制度）」等をわかりやすく解説するセミナーを開催します。…</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/careerweb/kigyo/seminar/ryouritusienn.html</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>2026-06-30 08:14:10</t>
         </is>
       </c>
     </row>
@@ -6378,7 +6410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6723,7 +6755,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>5万円</t>
@@ -6742,6 +6773,40 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>2026-06-27 08:21:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>仕事と育児・介護・治療の両立支援 助成金活用セミナー（終了しました）</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>更新日：2026年6月19日 実施内容 現在、「人口減少に伴う生産年齢人口の減少」、「仕事と育児や介護との両立など、働く方のニーズの多様化」に直面しています。こうした中、生産性の向上を図り、就業機会の拡大や意欲・能力を充分に発揮できる環境を作ることが重要な課題となっています。 本市では、働き方改革支援の観点から「両立支援等助成金（仕事と育児・介護の両立支援に取り組む事業主を応援する制度）」等をわかりやすく解説するセミナーを開催します。…</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/careerweb/kigyo/seminar/ryouritusienn.html</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-06-30 08:14:10</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7158,6 @@
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>大阪市は、家庭及び中小企業等の早期の省エネルギー化並びに再生可能エネルギーの導入拡大及び電力需給の安定化を図り、断熱窓及び省エネ設備等の導入加速により、大阪市の2030年度の温室効果ガス排出量削減目標達成に貢献することを目的とし補助金事業を実施します。実施にあたり、補助金の周知および円滑な活用につなげることを目的に説明会を開催します。説明会では申請にかかる注意点等をご理解いただき、申請時の不備等を減らし、事業者と行政双方の負担軽減を図…</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-06 08:18 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4655,8 +4655,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>更新日：2026年6月19日 実施内容 現在、「人口減少に伴う生産年齢人口の減少」、「仕事と育児や介護との両立など、働く方のニーズの多様化」に直面しています。こうした中、生産性の向上を図り、就業機会の拡大や意欲・能力を充分に発揮できる環境を作ることが重要な課題となっています。 本市では、働き方改革支援の観点から「両立支援等助成金（仕事と育児・介護の両立支援に取り組む事業主を応援する制度）」等をわかりやすく解説するセミナーを開催します。…</t>
@@ -4670,6 +4668,40 @@
       <c r="H112" t="inlineStr">
         <is>
           <t>2026-06-30 08:14:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>補助金・支援制度一覧</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>事業所向け再エネ電力利用促進事業 事業所向け省エネ設備等導入支援事業補助金【再エネ設備】 【堺エネルギー地産地消プロジェクト】建物の屋根に余剰電力活用型の太陽光発電設備を導入する事業者を募集します【令和8年度募集】 事業所向け省エネ設備等導入支援事業補助金 堺市スマートハウス化等支援事業 堺市ZEH支援事業 空気圧縮機・省エネアドバイザー派遣事業</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/gomi/ondanka/oshirase/hojokin_shien/index.html</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2026-07-06 08:15:40</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6792,8 +6824,6 @@
           <t>終了</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>更新日：2026年6月19日 実施内容 現在、「人口減少に伴う生産年齢人口の減少」、「仕事と育児や介護との両立など、働く方のニーズの多様化」に直面しています。こうした中、生産性の向上を図り、就業機会の拡大や意欲・能力を充分に発揮できる環境を作ることが重要な課題となっています。 本市では、働き方改革支援の観点から「両立支援等助成金（仕事と育児・介護の両立支援に取り組む事業主を応援する制度）」等をわかりやすく解説するセミナーを開催します。…</t>
@@ -6807,6 +6837,40 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-06-30 08:14:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>補助金・支援制度一覧</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>事業所向け再エネ電力利用促進事業 事業所向け省エネ設備等導入支援事業補助金【再エネ設備】 【堺エネルギー地産地消プロジェクト】建物の屋根に余剰電力活用型の太陽光発電設備を導入する事業者を募集します【令和8年度募集】 事業所向け省エネ設備等導入支援事業補助金 堺市スマートハウス化等支援事業 堺市ZEH支援事業 空気圧縮機・省エネアドバイザー派遣事業</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/gomi/ondanka/oshirase/hojokin_shien/index.html</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-07-06 08:15:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-07 08:24 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H113"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4687,8 +4687,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>事業所向け再エネ電力利用促進事業 事業所向け省エネ設備等導入支援事業補助金【再エネ設備】 【堺エネルギー地産地消プロジェクト】建物の屋根に余剰電力活用型の太陽光発電設備を導入する事業者を募集します【令和8年度募集】 事業所向け省エネ設備等導入支援事業補助金 堺市スマートハウス化等支援事業 堺市ZEH支援事業 空気圧縮機・省エネアドバイザー派遣事業</t>
@@ -4702,6 +4700,40 @@
       <c r="H113" t="inlineStr">
         <is>
           <t>2026-07-06 08:15:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>助成金・補助</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>公募中</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>ページ番号：91509513 西宮市障害者雇用奨励金 兵庫型奨学金返済支援制度 ワーク・ライフ・バランス助成金 求職者支援制度のお知らせ 2026年度介護職員初任者研修等受講費助成金の申請について（受付中） 本文ここまで</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kurashi/rodo/joseikin_hojo/index.html</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026-07-07 08:24:19</t>
         </is>
       </c>
     </row>
@@ -5713,7 +5745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6135,6 +6167,40 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>2026-06-23 08:45:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>助成金・補助</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>公募中</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ページ番号：91509513 西宮市障害者雇用奨励金 兵庫型奨学金返済支援制度 ワーク・ライフ・バランス助成金 求職者支援制度のお知らせ 2026年度介護職員初任者研修等受講費助成金の申請について（受付中） 本文ここまで</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kurashi/rodo/joseikin_hojo/index.html</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-07-07 08:24:19</t>
         </is>
       </c>
     </row>
@@ -6856,8 +6922,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>事業所向け再エネ電力利用促進事業 事業所向け省エネ設備等導入支援事業補助金【再エネ設備】 【堺エネルギー地産地消プロジェクト】建物の屋根に余剰電力活用型の太陽光発電設備を導入する事業者を募集します【令和8年度募集】 事業所向け省エネ設備等導入支援事業補助金 堺市スマートハウス化等支援事業 堺市ZEH支援事業 空気圧縮機・省エネアドバイザー派遣事業</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-10 08:27 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4719,8 +4719,6 @@
           <t>公募中</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>ページ番号：91509513 西宮市障害者雇用奨励金 兵庫型奨学金返済支援制度 ワーク・ライフ・バランス助成金 求職者支援制度のお知らせ 2026年度介護職員初任者研修等受講費助成金の申請について（受付中） 本文ここまで</t>
@@ -4734,6 +4732,44 @@
       <c r="H114" t="inlineStr">
         <is>
           <t>2026-07-07 08:24:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>森林の整備には里山林整備支援事業補助金をご利用ください</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>上限40万円</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月23日 ページ番号：40134936 森林は、水源のかん養、災害の防止、生物多様性の保全、地球温暖化防止等の多面的機能の発揮を通じて、市民が安全で安心して暮らせる社会の実現に重要な役割を果たしています。 民有林で手入れがなされずに荒廃し、放置された里山林が増加すると市民生活にも大きな影響を及ぼすことが考えられます。 住宅等に近い森林（民有林）にある危険木の除去や、地域住民による自主的な里山環境の維持保全を促し、森…</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kotsu/nogyo/shinrin/satoyamarinnhojokinn.html</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2026-07-10 08:27:41</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6186,8 +6222,6 @@
           <t>公募中</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>ページ番号：91509513 西宮市障害者雇用奨励金 兵庫型奨学金返済支援制度 ワーク・ライフ・バランス助成金 求職者支援制度のお知らせ 2026年度介護職員初任者研修等受講費助成金の申請について（受付中） 本文ここまで</t>
@@ -6201,6 +6235,44 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>2026-07-07 08:24:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>森林の整備には里山林整備支援事業補助金をご利用ください</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>上限40万円</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月23日 ページ番号：40134936 森林は、水源のかん養、災害の防止、生物多様性の保全、地球温暖化防止等の多面的機能の発揮を通じて、市民が安全で安心して暮らせる社会の実現に重要な役割を果たしています。 民有林で手入れがなされずに荒廃し、放置された里山林が増加すると市民生活にも大きな影響を及ぼすことが考えられます。 住宅等に近い森林（民有林）にある危険木の除去や、地域住民による自主的な里山環境の維持保全を促し、森…</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/kotsu/nogyo/shinrin/satoyamarinnhojokinn.html</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-07-10 08:27:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-18 08:07 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H115"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4751,7 +4751,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>上限40万円</t>
@@ -4770,6 +4769,48 @@
       <c r="H115" t="inlineStr">
         <is>
           <t>2026-07-10 08:27:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>西宮市移住支援金</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>※各年度の申請の受付期間は、4月1日から2月末日までです</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>60万円</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 ページ番号：29815917 西宮市では、市内でも人口減少が特に懸念される北部地域（西宮市支所設置条例における塩瀬支所及び山口支所の所管区域）への移住・定住の促進及び中小企業等における人手不足の解消に資するため、東京圏（埼玉県、千葉県、東京都及び神奈川県）から市の北部地域への移住者に対し、移住支援金を交付します。 要綱 ・西宮市移住支援金交付要綱（PDF：183KB） 交付金額について ・単身世帯の場合：6…</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/shisei/chihousousei/ijushien/ijushienkin.html</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026-07-18 08:06:49</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6254,7 +6295,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>上限40万円</t>
@@ -6273,6 +6313,48 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>2026-07-10 08:27:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>西宮市</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>西宮市移住支援金</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>※各年度の申請の受付期間は、4月1日から2月末日までです</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>60万円</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 ページ番号：29815917 西宮市では、市内でも人口減少が特に懸念される北部地域（西宮市支所設置条例における塩瀬支所及び山口支所の所管区域）への移住・定住の促進及び中小企業等における人手不足の解消に資するため、東京圏（埼玉県、千葉県、東京都及び神奈川県）から市の北部地域への移住者に対し、移住支援金を交付します。 要綱 ・西宮市移住支援金交付要綱（PDF：183KB） 交付金額について ・単身世帯の場合：6…</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.nishi.or.jp/shisei/chihousousei/ijushien/ijushienkin.html</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-07-18 08:06:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-20 08:09 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4811,6 +4811,40 @@
       <c r="H116" t="inlineStr">
         <is>
           <t>2026-07-18 08:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>補助金関係</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>児童福祉施設整備補助金関係 Jアラート受信情報 Jアラート受信情報一覧へ このページも読まれています 企業投資支援 補助金・支援制度一覧 情報が見つからないときは 堺市広報課 Twitter Twitterをスキップします。 Tweets by sakai_koho PC版を表示する スマートフォン版を表示する</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kosodate/hughug/kosodatekankyo/sonota/hojo_kin/index.html</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2026-07-20 08:06:19</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7089,6 +7123,40 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>2026-07-06 08:15:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>補助金関係</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>児童福祉施設整備補助金関係 Jアラート受信情報 Jアラート受信情報一覧へ このページも読まれています 企業投資支援 補助金・支援制度一覧 情報が見つからないときは 堺市広報課 Twitter Twitterをスキップします。 Tweets by sakai_koho PC版を表示する スマートフォン版を表示する</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kosodate/hughug/kosodatekankyo/sonota/hojo_kin/index.html</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-07-20 08:06:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-28 08:20 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4830,8 +4830,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>児童福祉施設整備補助金関係 Jアラート受信情報 Jアラート受信情報一覧へ このページも読まれています 企業投資支援 補助金・支援制度一覧 情報が見つからないときは 堺市広報課 Twitter Twitterをスキップします。 Tweets by sakai_koho PC版を表示する スマートフォン版を表示する</t>
@@ -4845,6 +4843,90 @@
       <c r="H117" t="inlineStr">
         <is>
           <t>2026-07-20 08:06:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>神戸市</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>神戸市内企業住宅手当等支援補助金～こうべ「住む×働く」若者応援補助金～</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>上限1万円</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>昨年度からの変更ポイント 「40歳未満」に対象を拡充！ 「2027年採用者」の補助を確約！採用面接時にお伝えいただけます。 就労者の住宅手当は、企業の福利厚生として就活生からのニーズが高く、企業での導入率も高くなっています。市内中小・中堅企業に勤務し、かつ市内に居住する従業員を対象に当該手当等の上乗せ支援を行います。 また、住民の高齢化傾向が強い地域（北区・長田区・須磨区・垂水区・西区及びその他の区の一部の小学校区）に居住する場合はさ…</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>https://www.city.kobe.lg.jp/a31812/jutakuteate.html</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>2026-07-28 08:20:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>神戸市</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>神戸市省エネ設備更新補助金</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>上限50万円</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>エネルギー価格高騰の影響を受ける市内事業者への支援として、「省エネ設備更新補助金」を実施します。 本補助金は、国の物価高対策（重点支援地方交付金）を活用した事業です。 お知らせ 第1期交付申請が予算上限に達したため、申請を締め切りました。 第2期は8月3日（月曜）10時00分より受付開始します 。 （交付申請をされた方へ）順次審査を行っております。結果通知まで今しばらくお待ちください。審査結果や不備補正のご連絡は、e-KOBEシステム…</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>https://www.city.kobe.lg.jp/a31812/kobe-syoene2026.html</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>2026-07-28 08:20:06</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5436,6 +5518,90 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>2026-05-04 02:15:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>神戸市</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>神戸市内企業住宅手当等支援補助金～こうべ「住む×働く」若者応援補助金～</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>上限1万円</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>昨年度からの変更ポイント 「40歳未満」に対象を拡充！ 「2027年採用者」の補助を確約！採用面接時にお伝えいただけます。 就労者の住宅手当は、企業の福利厚生として就活生からのニーズが高く、企業での導入率も高くなっています。市内中小・中堅企業に勤務し、かつ市内に居住する従業員を対象に当該手当等の上乗せ支援を行います。 また、住民の高齢化傾向が強い地域（北区・長田区・須磨区・垂水区・西区及びその他の区の一部の小学校区）に居住する場合はさ…</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.city.kobe.lg.jp/a31812/jutakuteate.html</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-07-28 08:20:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>神戸市</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>神戸市省エネ設備更新補助金</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>公募開始</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>上限50万円</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>エネルギー価格高騰の影響を受ける市内事業者への支援として、「省エネ設備更新補助金」を実施します。 本補助金は、国の物価高対策（重点支援地方交付金）を活用した事業です。 お知らせ 第1期交付申請が予算上限に達したため、申請を締め切りました。 第2期は8月3日（月曜）10時00分より受付開始します 。 （交付申請をされた方へ）順次審査を行っております。結果通知まで今しばらくお待ちください。審査結果や不備補正のご連絡は、e-KOBEシステム…</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.city.kobe.lg.jp/a31812/kobe-syoene2026.html</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-07-28 08:20:06</t>
         </is>
       </c>
     </row>
@@ -7142,8 +7308,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>児童福祉施設整備補助金関係 Jアラート受信情報 Jアラート受信情報一覧へ このページも読まれています 企業投資支援 補助金・支援制度一覧 情報が見つからないときは 堺市広報課 Twitter Twitterをスキップします。 Tweets by sakai_koho PC版を表示する スマートフォン版を表示する</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-07-30 08:13 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H119"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4927,6 +4927,86 @@
       <c r="H119" t="inlineStr">
         <is>
           <t>2026-07-28 08:20:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>堺市伝統産業異業種連携（商品開発・販路開拓）チャレンジ補助金</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>補助上限額は100万円</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 事業概要 この制度は、伝統産業事業者等が異なる業種の事業者と連携し、そのノウハウを活かして行う商品開発から販路開拓等まで一体的に取り組む事業に要する経費を補助することにより、伝統産業の振興を図ることを目的としています。 補助内容について 以下の内容は概要となりますので、補助内容の詳細は募集要領をご確認ください。 補助対象者 補助対象者は、以下の1、2、3のいずれかに該当する者とします。 伝統産業事業者（本市…</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/collabochallenge.html</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026-07-30 08:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>堺市伝統産業生産力強化支援補助金</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>） （5）直近の決算報告書の写し（個人の場合は、これに相当す</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>上限5000万円</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月27日 事業概要 この補助金は、伝統産業事業者が行う工場用建物の取得・改修や生産設備の購入・修繕、操業環境の改善、稀少道具類の購入・修理に要する経費を支援することにより、生産力を強化し、伝統産業の振興を図ることを目的としています。 補助内容について 以下の内容は概要となりますので、補助内容の詳細は募集要項をご確認ください。 補助対象者 補助対象者は、以下の1、2のいずれかに該当する者とします。 1.伝統産業事業者…</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/seisanryoku.html</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026-07-30 08:10:35</t>
         </is>
       </c>
     </row>
@@ -6862,7 +6942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7321,6 +7401,86 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>2026-07-20 08:06:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>堺市伝統産業異業種連携（商品開発・販路開拓）チャレンジ補助金</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>補助上限額は100万円</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 事業概要 この制度は、伝統産業事業者等が異なる業種の事業者と連携し、そのノウハウを活かして行う商品開発から販路開拓等まで一体的に取り組む事業に要する経費を補助することにより、伝統産業の振興を図ることを目的としています。 補助内容について 以下の内容は概要となりますので、補助内容の詳細は募集要領をご確認ください。 補助対象者 補助対象者は、以下の1、2、3のいずれかに該当する者とします。 伝統産業事業者（本市…</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/collabochallenge.html</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-07-30 08:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>堺市伝統産業生産力強化支援補助金</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>） （5）直近の決算報告書の写し（個人の場合は、これに相当す</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>上限5000万円</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月27日 事業概要 この補助金は、伝統産業事業者が行う工場用建物の取得・改修や生産設備の購入・修繕、操業環境の改善、稀少道具類の購入・修理に要する経費を支援することにより、生産力を強化し、伝統産業の振興を図ることを目的としています。 補助内容について 以下の内容は概要となりますので、補助内容の詳細は募集要項をご確認ください。 補助対象者 補助対象者は、以下の1、2のいずれかに該当する者とします。 1.伝統産業事業者…</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/dentosangyo/subsidy/seisanryoku.html</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-07-30 08:10:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-08-03 08:10 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4946,7 +4946,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
           <t>補助上限額は100万円</t>
@@ -5007,6 +5006,44 @@
       <c r="H121" t="inlineStr">
         <is>
           <t>2026-07-30 08:10:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>事業所向け省エネ設備等導入支援事業補助金</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>補助上限額90万円</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>ご案内 堺市内の事業所を対象に、省エネ設備などの導入費用の一部を支援します。 申請前に、 省エネルギー専門家による省エネ診断 が必須です。 補助対象設備の導入をご検討されている方は、まずはこちらにお問い合わせください。 事前相談の内容に応じて、申請方法や必要書類をご案内します。 ※申請に関する相談は申請期間外でも随時受付しています。 【問合せ先】 堺市役所 環境エネルギー課 電話：072-228-7548 メール： kanene@ci…</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/gomi/ondanka/shoene/jigyou_shoene_hojo/index.html</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026-08-03 08:07:37</t>
         </is>
       </c>
     </row>
@@ -6942,7 +6979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7420,7 +7457,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>補助上限額は100万円</t>
@@ -7481,6 +7517,44 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>2026-07-30 08:10:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>事業所向け省エネ設備等導入支援事業補助金</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>補助上限額90万円</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ご案内 堺市内の事業所を対象に、省エネ設備などの導入費用の一部を支援します。 申請前に、 省エネルギー専門家による省エネ診断 が必須です。 補助対象設備の導入をご検討されている方は、まずはこちらにお問い合わせください。 事前相談の内容に応じて、申請方法や必要書類をご案内します。 ※申請に関する相談は申請期間外でも随時受付しています。 【問合せ先】 堺市役所 環境エネルギー課 電話：072-228-7548 メール： kanene@ci…</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/gomi/ondanka/shoene/jigyou_shoene_hojo/index.html</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-08-03 08:07:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-08-04 08:20 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H122"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5025,7 +5025,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
           <t>補助上限額90万円</t>
@@ -5044,6 +5043,44 @@
       <c r="H122" t="inlineStr">
         <is>
           <t>2026-08-03 08:07:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>事業所向け省エネ設備等導入支援事業補助金【再エネ設備】</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>限度額90万円</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 ご案内 堺市内の事業所を対象に、再エネ設備（自家消費型太陽光発電設備）の導入費用の一部を支援します。 申請前に、 専門家による発電シミュレーション実施 が必須です。 導入をご検討されている方は、まずはこちらにお問い合わせください。 事前相談の内容に応じて、申請方法や必要書類をご案内します。 ※申請に関する相談は申請期間外でも随時受付しています。 【問合せ先】 堺市役所 環境エネルギー課 電話：072-228…</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/gomi/ondanka/shoene/jigyou_shoene_hojo/hojo_saiene.html</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026-08-04 08:16:47</t>
         </is>
       </c>
     </row>
@@ -6979,7 +7016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7536,7 +7573,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>補助上限額90万円</t>
@@ -7555,6 +7591,44 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>2026-08-03 08:07:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>事業所向け省エネ設備等導入支援事業補助金【再エネ設備】</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>限度額90万円</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 ご案内 堺市内の事業所を対象に、再エネ設備（自家消費型太陽光発電設備）の導入費用の一部を支援します。 申請前に、 専門家による発電シミュレーション実施 が必須です。 導入をご検討されている方は、まずはこちらにお問い合わせください。 事前相談の内容に応じて、申請方法や必要書類をご案内します。 ※申請に関する相談は申請期間外でも随時受付しています。 【問合せ先】 堺市役所 環境エネルギー課 電話：072-228…</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/kurashi/gomi/ondanka/shoene/jigyou_shoene_hojo/hojo_saiene.html</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-08-04 08:16:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-08-07 10:37 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5062,7 +5062,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
           <t>限度額90万円</t>
@@ -5081,6 +5080,78 @@
       <c r="H123" t="inlineStr">
         <is>
           <t>2026-08-04 08:16:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>中小企業向け補助金・総合支援サイト　ミラサポplus（経済産業省・中小企業庁）（外部リンク）</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>公募中</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>重要な お知らせ 2026年07月01日 中東情勢等を踏まえた中小企業・小規模事業者向け支援について 最新情報 一覧を見る 2026年08月04日 NEW 【補助金】成長加速化補助金（2次公募）の補助金交付候補者を採択 2026年08月03日 NEW 中小企業庁担当者に聞く「持続化補助金」 2026年07月31日 NEW 【省力化投資補助金（一般型）】令和8年熊本地震の被害を受けた熊本県内の事業者は第... 2026年07月29日 令…</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://mirasapo-plus.go.jp/</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:35:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>事業主のための雇用関係助成金（厚生労働省）（外部リンク）</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>ホーム &gt; 政策について &gt; 分野別の政策一覧 &gt; 雇用・労働 &gt; 雇用 &gt; 事業主の方のための雇用関係助成金 雇用・労働 事業主の方のための雇用関係助成金 お知らせ 2026（令和８）年７月17日 雇用関係助成金の添付書類標準化に関する アンケート を実施しています。（人事労務ソフトベンダ向け） 2023（令和５）年３月31日 生産性要件 は廃止になりました。 2022（令和４）年８月１日 雇用関係助成金の申請時、登記事項証明書の提…</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://www.mhlw.go.jp/stf/seisakunitsuite/bunya/koyou_roudou/koyou/kyufukin/index.html</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:35:06</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7681,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>限度額90万円</t>
@@ -8638,7 +8708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9255,6 +9325,78 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>2026-06-16 09:00:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>中小企業向け補助金・総合支援サイト　ミラサポplus（経済産業省・中小企業庁）（外部リンク）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>公募中</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>重要な お知らせ 2026年07月01日 中東情勢等を踏まえた中小企業・小規模事業者向け支援について 最新情報 一覧を見る 2026年08月04日 NEW 【補助金】成長加速化補助金（2次公募）の補助金交付候補者を採択 2026年08月03日 NEW 中小企業庁担当者に聞く「持続化補助金」 2026年07月31日 NEW 【省力化投資補助金（一般型）】令和8年熊本地震の被害を受けた熊本県内の事業者は第... 2026年07月29日 令…</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://mirasapo-plus.go.jp/</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:35:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>事業主のための雇用関係助成金（厚生労働省）（外部リンク）</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ホーム &gt; 政策について &gt; 分野別の政策一覧 &gt; 雇用・労働 &gt; 雇用 &gt; 事業主の方のための雇用関係助成金 雇用・労働 事業主の方のための雇用関係助成金 お知らせ 2026（令和８）年７月17日 雇用関係助成金の添付書類標準化に関する アンケート を実施しています。（人事労務ソフトベンダ向け） 2023（令和５）年３月31日 生産性要件 は廃止になりました。 2022（令和４）年８月１日 雇用関係助成金の申請時、登記事項証明書の提…</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.mhlw.go.jp/stf/seisakunitsuite/bunya/koyou_roudou/koyou/kyufukin/index.html</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:35:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-09-04 09:04 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5104,7 +5104,6 @@
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>重要な お知らせ 2026年07月01日 中東情勢等を踏まえた中小企業・小規模事業者向け支援について 最新情報 一覧を見る 2026年08月04日 NEW 【補助金】成長加速化補助金（2次公募）の補助金交付候補者を採択 2026年08月03日 NEW 中小企業庁担当者に聞く「持続化補助金」 2026年07月31日 NEW 【省力化投資補助金（一般型）】令和8年熊本地震の被害を受けた熊本県内の事業者は第... 2026年07月29日 令…</t>
@@ -5137,8 +5136,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>ホーム &gt; 政策について &gt; 分野別の政策一覧 &gt; 雇用・労働 &gt; 雇用 &gt; 事業主の方のための雇用関係助成金 雇用・労働 事業主の方のための雇用関係助成金 お知らせ 2026（令和８）年７月17日 雇用関係助成金の添付書類標準化に関する アンケート を実施しています。（人事労務ソフトベンダ向け） 2023（令和５）年３月31日 生産性要件 は廃止になりました。 2022（令和４）年８月１日 雇用関係助成金の申請時、登記事項証明書の提…</t>
@@ -5152,6 +5149,44 @@
       <c r="H125" t="inlineStr">
         <is>
           <t>2026-08-07 10:35:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>企業成長促進補助金（成長産業、特定重要物資・技術関連への投資）</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>50,000,000円</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 1 制度の趣旨 堺市では企業の本社機能や研究開発施設の投資を誘導するとともに、市内製造業等の成長産業、特定重要物資及び特定重要技術に係る投資を支援することにより、本市における雇用機会及び事業機会の拡大並びに産業集積の高度化、ひいては税源涵養や市内在住雇用者の増加を図ります。 2 制度の概要（成長産業、特定重要物資・技術関連への投資） 対象者 堺市内において、成長産業、特定重要物資又は特定重要技術に関する事業…</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/kigyoricchi/gp/seicho_hojo.html</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:01:28</t>
         </is>
       </c>
     </row>
@@ -7087,7 +7122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7699,6 +7734,44 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>2026-08-04 08:16:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>堺市</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>企業成長促進補助金（成長産業、特定重要物資・技術関連への投資）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>50,000,000円</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>更新日：2026年4月1日 1 制度の趣旨 堺市では企業の本社機能や研究開発施設の投資を誘導するとともに、市内製造業等の成長産業、特定重要物資及び特定重要技術に係る投資を支援することにより、本市における雇用機会及び事業機会の拡大並びに産業集積の高度化、ひいては税源涵養や市内在住雇用者の増加を図ります。 2 制度の概要（成長産業、特定重要物資・技術関連への投資） 対象者 堺市内において、成長産業、特定重要物資又は特定重要技術に関する事業…</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.city.sakai.lg.jp/sangyo/shienyuushi/kigyoricchi/gp/seicho_hojo.html</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:01:28</t>
         </is>
       </c>
     </row>
@@ -9349,7 +9422,6 @@
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>重要な お知らせ 2026年07月01日 中東情勢等を踏まえた中小企業・小規模事業者向け支援について 最新情報 一覧を見る 2026年08月04日 NEW 【補助金】成長加速化補助金（2次公募）の補助金交付候補者を採択 2026年08月03日 NEW 中小企業庁担当者に聞く「持続化補助金」 2026年07月31日 NEW 【省力化投資補助金（一般型）】令和8年熊本地震の被害を受けた熊本県内の事業者は第... 2026年07月29日 令…</t>
@@ -9382,8 +9454,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>ホーム &gt; 政策について &gt; 分野別の政策一覧 &gt; 雇用・労働 &gt; 雇用 &gt; 事業主の方のための雇用関係助成金 雇用・労働 事業主の方のための雇用関係助成金 お知らせ 2026（令和８）年７月17日 雇用関係助成金の添付書類標準化に関する アンケート を実施しています。（人事労務ソフトベンダ向け） 2023（令和５）年３月31日 生産性要件 は廃止になりました。 2022（令和４）年８月１日 雇用関係助成金の申請時、登記事項証明書の提…</t>

</xml_diff>

<commit_message>
chore(scrape): auto update 2026-09-10 09:12 JST
</commit_message>
<xml_diff>
--- a/data/grants.xlsx
+++ b/data/grants.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5168,7 +5168,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>50,000,000円</t>
@@ -5187,6 +5186,40 @@
       <c r="H126" t="inlineStr">
         <is>
           <t>2026-09-04 09:01:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>【地域経済振興室　企業振興担当】補助金関係書類等提出フォーム</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>手続き申込 ホーム 手続き説明 手続き説明 申込期間ではありません。 手続き名 【地域経済振興室 企業振興担当】 補助金関係書類等提出フォーム 説明 【地域経済振興室 企業振興担当宛】 に提出する、 補助金関係書類等 の提出用フォームです。 送受信の容量や添付方法に不安がある場合にも、御利用いただけます。 書類受付後、処理が完了までしばらくお待ちください。 提出書類等に関して確認事項がある場合は、企業振興担当から連絡いたします。 受付…</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>https://apply.e-tumo.jp/city-suita-osaka-u/offer/offerList_detail?tempSeq=32013</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026-09-10 09:10:28</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7786,6 @@
           <t>不明</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>50,000,000円</t>
@@ -8781,7 +8813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9467,6 +9499,40 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>2026-08-07 10:35:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>吹田市</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>【地域経済振興室　企業振興担当】補助金関係書類等提出フォーム</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>手続き申込 ホーム 手続き説明 手続き説明 申込期間ではありません。 手続き名 【地域経済振興室 企業振興担当】 補助金関係書類等提出フォーム 説明 【地域経済振興室 企業振興担当宛】 に提出する、 補助金関係書類等 の提出用フォームです。 送受信の容量や添付方法に不安がある場合にも、御利用いただけます。 書類受付後、処理が完了までしばらくお待ちください。 提出書類等に関して確認事項がある場合は、企業振興担当から連絡いたします。 受付…</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://apply.e-tumo.jp/city-suita-osaka-u/offer/offerList_detail?tempSeq=32013</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-09-10 09:10:28</t>
         </is>
       </c>
     </row>

</xml_diff>